<commit_message>
audit(phase3): resolve log loss formula bug, validate metrics, and regenerate corrected Phase 3 report artifacts
</commit_message>
<xml_diff>
--- a/phase3_results/ARGUS_Phase3_Results.xlsx
+++ b/phase3_results/ARGUS_Phase3_Results.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,6 +488,11 @@
           <t>PR_AUC</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Log_Loss</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -538,6 +543,9 @@
       <c r="L2" t="n">
         <v>0.1365601067550676</v>
       </c>
+      <c r="M2" t="n">
+        <v>9.803544050947078</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -588,6 +596,9 @@
       <c r="L3" t="n">
         <v>0.1365601067550676</v>
       </c>
+      <c r="M3" t="n">
+        <v>9.803544050947078</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -638,6 +649,9 @@
       <c r="L4" t="n">
         <v>0.2023143150123838</v>
       </c>
+      <c r="M4" t="n">
+        <v>0.912011338017033</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -688,6 +702,9 @@
       <c r="L5" t="n">
         <v>0.2023143150123838</v>
       </c>
+      <c r="M5" t="n">
+        <v>0.912011338017033</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -738,6 +755,9 @@
       <c r="L6" t="n">
         <v>0.1790305447640328</v>
       </c>
+      <c r="M6" t="n">
+        <v>4.517071071599526</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -788,6 +808,9 @@
       <c r="L7" t="n">
         <v>0.1790305447640328</v>
       </c>
+      <c r="M7" t="n">
+        <v>4.517071071599526</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -838,6 +861,9 @@
       <c r="L8" t="n">
         <v>0.1694631838115055</v>
       </c>
+      <c r="M8" t="n">
+        <v>1.217049886673418</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -888,6 +914,9 @@
       <c r="L9" t="n">
         <v>0.1694631838115055</v>
       </c>
+      <c r="M9" t="n">
+        <v>1.217049886673418</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -938,6 +967,9 @@
       <c r="L10" t="n">
         <v>0.558041405362643</v>
       </c>
+      <c r="M10" t="n">
+        <v>6.234225639607338</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -988,6 +1020,9 @@
       <c r="L11" t="n">
         <v>0.558041405362643</v>
       </c>
+      <c r="M11" t="n">
+        <v>6.234225639607338</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1038,6 +1073,9 @@
       <c r="L12" t="n">
         <v>0.181172001150594</v>
       </c>
+      <c r="M12" t="n">
+        <v>1.076163850258507</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1087,6 +1125,9 @@
       </c>
       <c r="L13" t="n">
         <v>0.181172001150594</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1.076163850258507</v>
       </c>
     </row>
   </sheetData>
@@ -1100,50 +1141,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Experiment_ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Training_Time_s</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Inference_Time_s</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>D1_D3_DANN</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>4.640429019927979</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.3673510551452637</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>D2_D3_DANN</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>3.877747058868408</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.3704030513763428</v>
+          <t>Runtimes loaded from checkpoints — see logs</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1347,7 +1359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1437,12 +1449,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Metrics Audit</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Independent validation completed 2026-08-19T22:43:11.488218 — Log Loss corrected from 0.0 to computed values</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Execution Timestamp</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-08-19T15:19:33.268218</t>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-19T22:43:11.488221</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1699,7 @@
         <v>0.1365601067550676</v>
       </c>
       <c r="X2" t="n">
-        <v>0</v>
+        <v>9.803544050947078</v>
       </c>
       <c r="Y2" t="n">
         <v>0.7560514411466094</v>
@@ -1767,7 +1791,7 @@
         <v>0.1365601067550676</v>
       </c>
       <c r="X3" t="n">
-        <v>0</v>
+        <v>9.803544050947078</v>
       </c>
       <c r="Y3" t="n">
         <v>0.7560514411466094</v>
@@ -1859,13 +1883,13 @@
         <v>0.2023143150123838</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>0.912011338017033</v>
       </c>
       <c r="Y4" t="n">
         <v>0.2223956177526085</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.2104860995691225</v>
+        <v>0.2104860995691226</v>
       </c>
     </row>
     <row r="5">
@@ -1951,13 +1975,13 @@
         <v>0.2023143150123838</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>0.912011338017033</v>
       </c>
       <c r="Y5" t="n">
         <v>0.2223956177526085</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.2104860995691225</v>
+        <v>0.2104860995691226</v>
       </c>
     </row>
     <row r="6">
@@ -2043,13 +2067,13 @@
         <v>0.1790305447640328</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>4.517071071599526</v>
       </c>
       <c r="Y6" t="n">
         <v>0.7508616313568289</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.7579735330644249</v>
+        <v>0.7579735330644247</v>
       </c>
     </row>
     <row r="7">
@@ -2135,13 +2159,13 @@
         <v>0.1790305447640328</v>
       </c>
       <c r="X7" t="n">
-        <v>0</v>
+        <v>4.517071071599526</v>
       </c>
       <c r="Y7" t="n">
         <v>0.7508616313568289</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.7579735330644249</v>
+        <v>0.7579735330644247</v>
       </c>
     </row>
     <row r="8">
@@ -2227,7 +2251,7 @@
         <v>0.1694631838115055</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>1.217049886673418</v>
       </c>
       <c r="Y8" t="n">
         <v>0.4545462811994256</v>
@@ -2319,7 +2343,7 @@
         <v>0.1694631838115055</v>
       </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>1.217049886673418</v>
       </c>
       <c r="Y9" t="n">
         <v>0.4545462811994256</v>
@@ -2411,13 +2435,13 @@
         <v>0.558041405362643</v>
       </c>
       <c r="X10" t="n">
-        <v>0</v>
+        <v>6.234225639607338</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.7508159875869751</v>
+        <v>0.7508160767553164</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.7558154422860009</v>
+        <v>0.7558154973519743</v>
       </c>
     </row>
     <row r="11">
@@ -2503,13 +2527,13 @@
         <v>0.558041405362643</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>6.234225639607338</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.7508159875869751</v>
+        <v>0.7508160767553164</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.7558154422860009</v>
+        <v>0.7558154973519743</v>
       </c>
     </row>
     <row r="12">
@@ -2595,13 +2619,13 @@
         <v>0.181172001150594</v>
       </c>
       <c r="X12" t="n">
-        <v>0</v>
+        <v>1.076163850258507</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.3321532607078552</v>
+        <v>0.3321532684412174</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.3301523891051648</v>
+        <v>0.330152424662924</v>
       </c>
     </row>
     <row r="13">
@@ -2687,13 +2711,13 @@
         <v>0.181172001150594</v>
       </c>
       <c r="X13" t="n">
-        <v>0</v>
+        <v>1.076163850258507</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.3321532607078552</v>
+        <v>0.3321532684412174</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.3301523891051648</v>
+        <v>0.330152424662924</v>
       </c>
     </row>
   </sheetData>
@@ -2760,7 +2784,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>D1_D3_BASELINE_UNCALIB</t>
+          <t>D1_D3_BASELINE</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -2791,7 +2815,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>D1_D3_BASELINE_CALIB</t>
+          <t>D1_D3_BASELINE_CALIBRATED</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2822,7 +2846,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>D2_D3_BASELINE_UNCALIB</t>
+          <t>D2_D3_BASELINE</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2853,7 +2877,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>D2_D3_BASELINE_CALIB</t>
+          <t>D2_D3_BASELINE_CALIBRATED</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2884,7 +2908,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>D1_D3_CORAL_UNCALIB</t>
+          <t>D1_D3_CORAL</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2915,7 +2939,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>D1_D3_CORAL_CALIB</t>
+          <t>D1_D3_CORAL_CALIBRATED</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2946,7 +2970,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>D2_D3_CORAL_UNCALIB</t>
+          <t>D2_D3_CORAL</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2977,7 +3001,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>D2_D3_CORAL_CALIB</t>
+          <t>D2_D3_CORAL_CALIBRATED</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -3008,7 +3032,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>D1_D3_DANN_UNCALIB</t>
+          <t>D1_D3_DANN</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -3039,7 +3063,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>D1_D3_DANN_CALIB</t>
+          <t>D1_D3_DANN_CALIBRATED</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -3070,7 +3094,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>D2_D3_DANN_UNCALIB</t>
+          <t>D2_D3_DANN</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -3101,7 +3125,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>D2_D3_DANN_CALIB</t>
+          <t>D2_D3_DANN_CALIBRATED</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -4000,13 +4024,13 @@
         <v>0.6299999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2486601637896405</v>
+        <v>0.2486601637896404</v>
       </c>
       <c r="F2" t="n">
         <v>0.2292214165848716</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9922745765034983</v>
+        <v>0.9922745765034984</v>
       </c>
       <c r="H2" t="n">
         <v>0.3724131480647933</v>
@@ -4039,25 +4063,25 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9699999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="E3" t="n">
-        <v>0.248675560183805</v>
+        <v>0.2486755601838049</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2292336188199535</v>
+        <v>0.2292336188199534</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9923431084861285</v>
+        <v>0.9923431084861284</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3724340793082566</v>
+        <v>0.3724340793082565</v>
       </c>
       <c r="I3" t="n">
         <v>0.5127679972048077</v>
       </c>
       <c r="J3" t="n">
-        <v>0.06522118808773511</v>
+        <v>0.0652211880877351</v>
       </c>
       <c r="K3" t="n">
         <v>0.5436945663672488</v>
@@ -4090,16 +4114,16 @@
         <v>0.2295603785689057</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9920814409160857</v>
+        <v>0.9920814409160856</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3728467501937545</v>
+        <v>0.3728467501937544</v>
       </c>
       <c r="I4" t="n">
         <v>0.5136571221159721</v>
       </c>
       <c r="J4" t="n">
-        <v>0.06782511973882797</v>
+        <v>0.0678251197388279</v>
       </c>
       <c r="K4" t="n">
         <v>0.4932073986761365</v>
@@ -4126,13 +4150,13 @@
         <v>0.6499999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2486741605116082</v>
+        <v>0.2486741605116081</v>
       </c>
       <c r="F5" t="n">
         <v>0.2292332889105086</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9923431084861285</v>
+        <v>0.9923431084861284</v>
       </c>
       <c r="H5" t="n">
         <v>0.3724336438895559</v>
@@ -4168,13 +4192,13 @@
         <v>0.5299999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2486741605116082</v>
+        <v>0.2486741605116081</v>
       </c>
       <c r="F6" t="n">
         <v>0.2292332889105086</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9923431084861285</v>
+        <v>0.9923431084861284</v>
       </c>
       <c r="H6" t="n">
         <v>0.3724336438895559</v>

</xml_diff>